<commit_message>
Update code with new data
</commit_message>
<xml_diff>
--- a/Data/All_strains_SCStimes.xlsx
+++ b/Data/All_strains_SCStimes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kienphan/WorkingSpace/ResearchProjs/ChromosomeSegeation/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7816AEB7-2A6B-324E-B39A-50296E2726FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4DA8B6F-6B58-9042-AB37-D6980AB479D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="33">
   <si>
     <t>wildtype12</t>
   </si>
@@ -113,6 +113,18 @@
   <si>
     <t>degRadeAPC32</t>
   </si>
+  <si>
+    <t>mis4N2_12</t>
+  </si>
+  <si>
+    <t>-108.5</t>
+  </si>
+  <si>
+    <t>-73.5</t>
+  </si>
+  <si>
+    <t>-59.5</t>
+  </si>
 </sst>
 </file>
 
@@ -168,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -187,6 +199,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -403,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J1000"/>
+  <dimension ref="A1:K1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
@@ -414,10 +429,11 @@
     <col min="7" max="7" width="25.83203125" style="8" customWidth="1"/>
     <col min="8" max="8" width="25.83203125" style="6" customWidth="1"/>
     <col min="9" max="10" width="24.6640625" customWidth="1"/>
-    <col min="11" max="26" width="8.6640625" customWidth="1"/>
+    <col min="11" max="11" width="28.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -448,8 +464,11 @@
       <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" s="2">
         <v>-3.5</v>
       </c>
@@ -480,8 +499,11 @@
       <c r="J2" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="K2" s="9">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" s="2">
         <v>0</v>
       </c>
@@ -512,8 +534,11 @@
       <c r="J3" s="3">
         <v>41</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="K3" s="9">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" s="2">
         <v>0</v>
       </c>
@@ -544,8 +569,11 @@
       <c r="J4" s="3">
         <v>111</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="K4" s="9">
+        <v>-70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" s="2">
         <v>3.5</v>
       </c>
@@ -576,8 +604,11 @@
       <c r="J5" s="3">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5" s="9">
+        <v>-28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" s="2">
         <v>21</v>
       </c>
@@ -608,8 +639,11 @@
       <c r="J6" s="3">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" spans="1:10">
+      <c r="K6" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" s="2">
         <v>10.5</v>
       </c>
@@ -640,8 +674,11 @@
       <c r="J7" s="3">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:10">
+      <c r="K7" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" s="2">
         <v>-38.5</v>
       </c>
@@ -672,8 +709,11 @@
       <c r="J8" s="3">
         <v>-15</v>
       </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="K8" s="9">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" s="2">
         <v>21</v>
       </c>
@@ -704,8 +744,11 @@
       <c r="J9" s="3">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:10">
+      <c r="K9" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" s="2">
         <v>-59.5</v>
       </c>
@@ -736,8 +779,11 @@
       <c r="J10" s="3">
         <v>-57</v>
       </c>
-    </row>
-    <row r="11" spans="1:10">
+      <c r="K10" s="9">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" s="2">
         <v>-31.5</v>
       </c>
@@ -768,8 +814,11 @@
       <c r="J11" s="3">
         <v>14</v>
       </c>
-    </row>
-    <row r="12" spans="1:10">
+      <c r="K11" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" s="2">
         <v>24.5</v>
       </c>
@@ -800,8 +849,11 @@
       <c r="J12" s="3">
         <v>48</v>
       </c>
-    </row>
-    <row r="13" spans="1:10">
+      <c r="K12" s="9">
+        <v>-35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" s="2">
         <v>3.5</v>
       </c>
@@ -832,8 +884,11 @@
       <c r="J13" s="3">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:10">
+      <c r="K13" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" s="2">
         <v>21</v>
       </c>
@@ -864,8 +919,11 @@
       <c r="J14" s="3">
         <v>48</v>
       </c>
-    </row>
-    <row r="15" spans="1:10">
+      <c r="K14" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15" s="2">
         <v>3.5</v>
       </c>
@@ -896,8 +954,11 @@
       <c r="J15" s="3">
         <v>76</v>
       </c>
-    </row>
-    <row r="16" spans="1:10">
+      <c r="K15" s="9">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16" s="2">
         <v>-49</v>
       </c>
@@ -928,8 +989,11 @@
       <c r="J16" s="3">
         <v>105</v>
       </c>
-    </row>
-    <row r="17" spans="1:10">
+      <c r="K16" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17" s="2">
         <v>3.5</v>
       </c>
@@ -960,8 +1024,11 @@
       <c r="J17" s="3">
         <v>125</v>
       </c>
-    </row>
-    <row r="18" spans="1:10">
+      <c r="K17" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
       <c r="A18" s="2">
         <v>-7</v>
       </c>
@@ -992,8 +1059,11 @@
       <c r="J18" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:10">
+      <c r="K18" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19" s="2">
         <v>7</v>
       </c>
@@ -1024,8 +1094,11 @@
       <c r="J19" s="3">
         <v>104</v>
       </c>
-    </row>
-    <row r="20" spans="1:10">
+      <c r="K19" s="9">
+        <v>-28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" s="2">
         <v>56</v>
       </c>
@@ -1056,8 +1129,11 @@
       <c r="J20" s="3">
         <v>69</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K20" s="9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1">
       <c r="A21" s="2">
         <v>17.5</v>
       </c>
@@ -1088,8 +1164,11 @@
       <c r="J21" s="3">
         <v>-50</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K21" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1120,8 +1199,11 @@
       <c r="J22" s="3">
         <v>41</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K22" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1">
       <c r="A23" s="2">
         <v>-14</v>
       </c>
@@ -1152,8 +1234,11 @@
       <c r="J23" s="3">
         <v>76</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K23" s="9">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1">
       <c r="A24" s="2">
         <v>3.5</v>
       </c>
@@ -1184,8 +1269,11 @@
       <c r="J24" s="3">
         <v>272</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K24" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1">
       <c r="A25" s="2">
         <v>-49</v>
       </c>
@@ -1216,8 +1304,11 @@
       <c r="J25" s="3">
         <v>62</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K25" s="9">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1">
       <c r="A26" s="2">
         <v>-14</v>
       </c>
@@ -1248,8 +1339,11 @@
       <c r="J26" s="3">
         <v>-29</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K26" s="9">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" customHeight="1">
       <c r="A27" s="2">
         <v>-56</v>
       </c>
@@ -1280,8 +1374,11 @@
       <c r="J27" s="3">
         <v>55</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K27" s="9">
+        <v>-56</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="15.75" customHeight="1">
       <c r="A28" s="2">
         <v>17.5</v>
       </c>
@@ -1312,8 +1409,11 @@
       <c r="J28" s="3">
         <v>26</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K28" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="15.75" customHeight="1">
       <c r="A29" s="2">
         <v>24.5</v>
       </c>
@@ -1344,8 +1444,11 @@
       <c r="J29" s="3">
         <v>69</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K29" s="9">
+        <v>-28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="15.75" customHeight="1">
       <c r="A30" s="2">
         <v>6.8150000000000004</v>
       </c>
@@ -1376,8 +1479,11 @@
       <c r="J30" s="3">
         <v>27</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K30" s="9">
+        <v>-28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="15.75" customHeight="1">
       <c r="A31" s="2">
         <v>-15.311999999999999</v>
       </c>
@@ -1408,8 +1514,11 @@
       <c r="J31" s="3">
         <v>27</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K31" s="9">
+        <v>-28</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="15.75" customHeight="1">
       <c r="A32" s="2">
         <v>13.006</v>
       </c>
@@ -1440,8 +1549,11 @@
       <c r="J32" s="3">
         <v>34</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K32" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" customHeight="1">
       <c r="A33" s="2">
         <v>5.8970000000000002</v>
       </c>
@@ -1472,8 +1584,11 @@
       <c r="J33" s="3">
         <v>90</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K33" s="9">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="15.75" customHeight="1">
       <c r="A34" s="2">
         <v>-15.108000000000001</v>
       </c>
@@ -1504,8 +1619,11 @@
       <c r="J34" s="3">
         <v>13</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K34" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="15.75" customHeight="1">
       <c r="A35" s="2">
         <v>-50.48</v>
       </c>
@@ -1536,8 +1654,11 @@
       <c r="J35" s="3">
         <v>-57</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K35" s="9">
+        <v>-161</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="15.75" customHeight="1">
       <c r="A36" s="2">
         <v>-1.1121000000000001</v>
       </c>
@@ -1568,8 +1689,11 @@
       <c r="J36" s="3">
         <v>125</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K36" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="15.75" customHeight="1">
       <c r="A37" s="2">
         <v>-57.120100000000001</v>
       </c>
@@ -1600,8 +1724,11 @@
       <c r="J37" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K37" s="9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="15.75" customHeight="1">
       <c r="A38" s="2">
         <v>-15.071999999999999</v>
       </c>
@@ -1632,8 +1759,11 @@
       <c r="J38" s="3">
         <v>20</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K38" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="15.75" customHeight="1">
       <c r="A39" s="2">
         <v>-15.122</v>
       </c>
@@ -1664,8 +1794,11 @@
       <c r="J39" s="3">
         <v>26</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K39" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="15.75" customHeight="1">
       <c r="A40" s="2">
         <v>-1.7130000000000001</v>
       </c>
@@ -1696,8 +1829,11 @@
       <c r="J40" s="3">
         <v>14</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K40" s="9">
+        <v>-56</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="15.75" customHeight="1">
       <c r="A41" s="2">
         <v>26.914000000000001</v>
       </c>
@@ -1728,8 +1864,11 @@
       <c r="J41" s="3">
         <v>118</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K41" s="9">
+        <v>-35</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="15.75" customHeight="1">
       <c r="A42" s="2">
         <v>-1.0089999999999999</v>
       </c>
@@ -1760,8 +1899,11 @@
       <c r="J42" s="3">
         <v>55</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K42" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="15.75" customHeight="1">
       <c r="A43" s="2">
         <v>40.880000000000003</v>
       </c>
@@ -1792,8 +1934,11 @@
       <c r="J43" s="3">
         <v>41</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K43" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="15.75" customHeight="1">
       <c r="A44" s="2">
         <v>-1.1119000000000001</v>
       </c>
@@ -1824,8 +1969,11 @@
       <c r="J44" s="3">
         <v>62</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K44" s="9">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="15.75" customHeight="1">
       <c r="A45" s="2">
         <v>-8.1137999999999995</v>
       </c>
@@ -1856,8 +2004,11 @@
       <c r="J45" s="3">
         <v>27</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K45" s="9">
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1">
       <c r="A46" s="2">
         <v>-10.315899999999999</v>
       </c>
@@ -1888,8 +2039,11 @@
       <c r="J46" s="3">
         <v>42</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K46" s="9">
+        <v>-49</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" customHeight="1">
       <c r="A47" s="2">
         <v>-1.1079000000000001</v>
       </c>
@@ -1920,8 +2074,11 @@
       <c r="J47" s="3">
         <v>-7</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K47" s="9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="15.75" customHeight="1">
       <c r="A48" s="2">
         <v>-1.01</v>
       </c>
@@ -1952,8 +2109,11 @@
       <c r="J48" s="3">
         <v>28</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K48" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="15.75" customHeight="1">
       <c r="A49" s="2">
         <v>-1.1111</v>
       </c>
@@ -1984,8 +2144,11 @@
       <c r="J49" s="3">
         <v>-29</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K49" s="9">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="15.75" customHeight="1">
       <c r="A50" s="2">
         <v>5.9669999999999996</v>
       </c>
@@ -2016,8 +2179,11 @@
       <c r="J50" s="3">
         <v>34</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K50" s="9">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="15.75" customHeight="1">
       <c r="A51" s="2">
         <v>12.923999999999999</v>
       </c>
@@ -2048,8 +2214,11 @@
       <c r="J51" s="3">
         <v>251</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K51" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="15.75" customHeight="1">
       <c r="A52" s="2">
         <v>19.974</v>
       </c>
@@ -2080,8 +2249,11 @@
       <c r="J52" s="3">
         <v>13</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K52" s="9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="15.75" customHeight="1">
       <c r="A53" s="2">
         <v>-1.0569999999999999</v>
       </c>
@@ -2112,8 +2284,11 @@
       <c r="J53" s="3">
         <v>104</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K53" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="15.75" customHeight="1">
       <c r="A54" s="2">
         <v>-29.1069</v>
       </c>
@@ -2144,8 +2319,11 @@
       <c r="J54" s="3">
         <v>62</v>
       </c>
-    </row>
-    <row r="55" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K54" s="9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="15.75" customHeight="1">
       <c r="A55" s="2">
         <v>-1.099</v>
       </c>
@@ -2176,8 +2354,11 @@
       <c r="J55" s="3">
         <v>111</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K55" s="9">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="15.75" customHeight="1">
       <c r="A56" s="2">
         <v>5.9131</v>
       </c>
@@ -2208,8 +2389,11 @@
       <c r="J56" s="3">
         <v>-15</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K56" s="9">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="15.75" customHeight="1">
       <c r="A57" s="2">
         <v>-15.077999999999999</v>
       </c>
@@ -2240,8 +2424,11 @@
       <c r="J57" s="3">
         <v>63</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K57" s="9">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="15.75" customHeight="1">
       <c r="A58" s="2">
         <v>-8.08</v>
       </c>
@@ -2272,8 +2459,11 @@
       <c r="J58" s="3">
         <v>-29</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K58" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="15.75" customHeight="1">
       <c r="A59" s="2">
         <v>-1.0049999999999999</v>
       </c>
@@ -2304,8 +2494,11 @@
       <c r="J59" s="3">
         <v>34</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K59" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="15.75" customHeight="1">
       <c r="A60" s="2">
         <v>5.8939000000000004</v>
       </c>
@@ -2336,8 +2529,11 @@
       <c r="J60" s="3">
         <v>251</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K60" s="9">
+        <v>-28</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="15.75" customHeight="1">
       <c r="A61" s="2">
         <v>5.9099000000000004</v>
       </c>
@@ -2368,8 +2564,11 @@
       <c r="J61" s="3">
         <v>13</v>
       </c>
-    </row>
-    <row r="62" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K61" s="9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="15.75" customHeight="1">
       <c r="A62" s="2">
         <v>-1.099</v>
       </c>
@@ -2400,8 +2599,11 @@
       <c r="J62" s="3">
         <v>104</v>
       </c>
-    </row>
-    <row r="63" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K62" s="9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="15.75" customHeight="1">
       <c r="A63" s="2">
         <v>-1.0089999999999999</v>
       </c>
@@ -2432,8 +2634,11 @@
       <c r="J63" s="3">
         <v>62</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K63" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="15.75" customHeight="1">
       <c r="A64" s="2">
         <v>-15.023899999999999</v>
       </c>
@@ -2462,8 +2667,11 @@
       <c r="J64" s="3">
         <v>111</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K64" s="9">
+        <v>-70</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="15.75" customHeight="1">
       <c r="A65" s="2">
         <v>-8.0061</v>
       </c>
@@ -2492,8 +2700,11 @@
       <c r="J65" s="3">
         <v>-15</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K65" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="15.75" customHeight="1">
       <c r="A66" s="2">
         <v>-19.818999999999999</v>
       </c>
@@ -2522,8 +2733,11 @@
       <c r="J66" s="3">
         <v>63</v>
       </c>
-    </row>
-    <row r="67" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K66" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="15.75" customHeight="1">
       <c r="A67" s="2">
         <v>5.9779999999999998</v>
       </c>
@@ -2552,8 +2766,11 @@
       <c r="J67" s="3">
         <v>41</v>
       </c>
-    </row>
-    <row r="68" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K67" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="15.75" customHeight="1">
       <c r="A68" s="2">
         <v>9.5178999999999991</v>
       </c>
@@ -2582,8 +2799,11 @@
       <c r="J68" s="3">
         <v>62</v>
       </c>
-    </row>
-    <row r="69" spans="1:10" ht="15.75" customHeight="1">
+      <c r="K68" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="15.75" customHeight="1">
       <c r="A69" s="2">
         <v>12.99</v>
       </c>
@@ -2611,7 +2831,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="15.75" customHeight="1">
+    <row r="70" spans="1:11" ht="15.75" customHeight="1">
       <c r="A70" s="2">
         <v>-22.145</v>
       </c>
@@ -2639,7 +2859,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="15.75" customHeight="1">
+    <row r="71" spans="1:11" ht="15.75" customHeight="1">
       <c r="A71" s="2">
         <v>-14.3348</v>
       </c>
@@ -2667,7 +2887,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="15.75" customHeight="1">
+    <row r="72" spans="1:11" ht="15.75" customHeight="1">
       <c r="A72" s="2">
         <v>-15.008100000000001</v>
       </c>
@@ -2695,7 +2915,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="15.75" customHeight="1">
+    <row r="73" spans="1:11" ht="15.75" customHeight="1">
       <c r="A73" s="2">
         <v>-8.0120000000000005</v>
       </c>
@@ -2723,7 +2943,7 @@
         <v>-78</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="15.75" customHeight="1">
+    <row r="74" spans="1:11" ht="15.75" customHeight="1">
       <c r="A74" s="2">
         <v>-29.009</v>
       </c>
@@ -2751,7 +2971,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="15.75" customHeight="1">
+    <row r="75" spans="1:11" ht="15.75" customHeight="1">
       <c r="A75" s="2">
         <v>-8.0719999999999992</v>
       </c>
@@ -2779,7 +2999,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="15.75" customHeight="1">
+    <row r="76" spans="1:11" ht="15.75" customHeight="1">
       <c r="A76" s="2">
         <v>5.9729999999999999</v>
       </c>
@@ -2807,7 +3027,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="15.75" customHeight="1">
+    <row r="77" spans="1:11" ht="15.75" customHeight="1">
       <c r="A77" s="2">
         <v>5.9790000000000001</v>
       </c>
@@ -2835,7 +3055,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="15.75" customHeight="1">
+    <row r="78" spans="1:11" ht="15.75" customHeight="1">
       <c r="A78" s="2">
         <v>12.996</v>
       </c>
@@ -2863,7 +3083,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="15.75" customHeight="1">
+    <row r="79" spans="1:11" ht="15.75" customHeight="1">
       <c r="A79" s="2">
         <v>-1.0049999999999999</v>
       </c>
@@ -2891,7 +3111,7 @@
         <v>-22</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="15.75" customHeight="1">
+    <row r="80" spans="1:11" ht="15.75" customHeight="1">
       <c r="A80" s="2">
         <v>-15.0229</v>
       </c>

</xml_diff>